<commit_message>
Sheet2: logical reasoning is Logical deduction, SuperWEIRD Math keeps 3 skills
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DTbm6a7iHNzz2Nb3WUHdpr
</commit_message>
<xml_diff>
--- a/scripts/games-final.xlsx
+++ b/scripts/games-final.xlsx
@@ -18216,8 +18216,10 @@
       <c r="B19" s="20" t="s">
         <v>432</v>
       </c>
-      <c r="C19" s="19" t="s">
-        <v>436</v>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Strategic planning, Logical deduction</t>
+        </is>
       </c>
       <c r="D19" s="19" t="s">
         <v>307</v>
@@ -18790,8 +18792,10 @@
       <c r="B33" s="20" t="s">
         <v>513</v>
       </c>
-      <c r="C33" s="19" t="s">
-        <v>298</v>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arithmetic, Logical deduction</t>
+        </is>
       </c>
       <c r="D33" s="19" t="s">
         <v>44</v>
@@ -19282,8 +19286,10 @@
       <c r="B45" s="20" t="s">
         <v>546</v>
       </c>
-      <c r="C45" s="19" t="s">
-        <v>298</v>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arithmetic, Logical deduction</t>
+        </is>
       </c>
       <c r="D45" s="19" t="s">
         <v>29</v>
@@ -19651,8 +19657,10 @@
       <c r="B54" s="20" t="s">
         <v>570</v>
       </c>
-      <c r="C54" s="19" t="s">
-        <v>439</v>
+      <c r="C54" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Systems thinking, strategic planning, arithmetic</t>
+        </is>
       </c>
       <c r="D54" s="19" t="s">
         <v>87</v>

</xml_diff>